<commit_message>
Fix: student load subject dropdown now shows only assigned subjects per instructor
</commit_message>
<xml_diff>
--- a/BackEnd/schedule_output.xlsx
+++ b/BackEnd/schedule_output.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faculty Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Faculty Schedule'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Faculty Schedule'!$A$1:$G$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -94,13 +94,13 @@
     <font>
       <name val="Liberation Sans"/>
       <b val="1"/>
-      <color rgb="00475569"/>
+      <color rgb="001E40AF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Liberation Sans"/>
       <b val="1"/>
-      <color rgb="001E40AF"/>
+      <color rgb="00475569"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -327,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -368,10 +368,13 @@
     <xf numFmtId="49" fontId="11" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="12" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="12" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="9" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -743,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -835,14 +838,14 @@
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>JERAHMEEL CANTOS</t>
+          <t>BRYAN PADERES</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Total: 1 hr   |   Lecture: 1 hr (1 slot)   |   Laboratory: 0 hrs (0 slots)</t>
+          <t>Total: 5 hrs   |   Lecture: 3 hrs (3 slots)   |   Laboratory: 2 hrs (2 slots)</t>
         </is>
       </c>
     </row>
@@ -891,14 +894,21 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SIA
-[3A]
-Room 1
+          <t>301
+[2c]
+Room 4
 [Lecture]</t>
         </is>
       </c>
       <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>IT  1o1
+[3a]
+Lab A
+[Laboratory]</t>
+        </is>
+      </c>
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
@@ -910,7 +920,14 @@
         </is>
       </c>
       <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="n"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>302
+[1b]
+Room 4
+[Lecture]</t>
+        </is>
+      </c>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
@@ -922,11 +939,25 @@
           <t>10:00 AM - 11:00 AM</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n"/>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>166
+[4a]
+Room 1
+[Lecture]</t>
+        </is>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>capstone1
+[3c]
+Lab C
+[Laboratory]</t>
+        </is>
+      </c>
       <c r="G15" s="15" t="n"/>
     </row>
     <row r="16" ht="46" customHeight="1">
@@ -1047,17 +1078,17 @@
       <c r="G24" s="15" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Laboratory</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Lecture Room</t>
         </is>
@@ -1068,13 +1099,13 @@
       <c r="G25" s="1" t="n"/>
     </row>
     <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="19" t="n"/>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
-      <c r="G26" s="19" t="n"/>
+      <c r="A26" s="20" t="n"/>
+      <c r="B26" s="20" t="n"/>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="20" t="n"/>
+      <c r="F26" s="20" t="n"/>
+      <c r="G26" s="20" t="n"/>
     </row>
     <row r="27" ht="10" customHeight="1">
       <c r="A27" s="1" t="n"/>
@@ -1085,15 +1116,1049 @@
       <c r="F27" s="1" t="n"/>
       <c r="G27" s="1" t="n"/>
     </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>DE JUAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Total: 1 hr   |   Lecture: 1 hr (1 slot)   |   Laboratory: 0 hrs (0 slots)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="46" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>8:00 AM - 9:00 AM</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="15" t="n"/>
+    </row>
+    <row r="32" ht="46" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>9:00 AM - 10:00 AM</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="46" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>10:00 AM - 11:00 AM</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="15" t="n"/>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>11:00 AM - 12:00 PM</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+    </row>
+    <row r="35" ht="46" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="15" t="n"/>
+    </row>
+    <row r="36" ht="46" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>1:00 PM - 2:00 PM</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15" t="n"/>
+      <c r="G36" s="15" t="n"/>
+    </row>
+    <row r="37" ht="46" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>2:00 PM - 3:00 PM</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="15" t="n"/>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>3:00 PM - 4:00 PM</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="15" t="n"/>
+    </row>
+    <row r="39" ht="46" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>4:00 PM - 5:00 PM</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="15" t="n"/>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>5:00 PM - 6:00 PM</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="15" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="15" t="n"/>
+      <c r="F40" s="15" t="n"/>
+      <c r="G40" s="15" t="n"/>
+    </row>
+    <row r="41" ht="46" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>IT 101
+[1C]
+Room 5
+[Lecture]</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="15" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="15" t="n"/>
+    </row>
+    <row r="42" ht="46" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>7:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Laboratory</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lecture Room</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="n"/>
+      <c r="E43" s="1" t="n"/>
+      <c r="F43" s="1" t="n"/>
+      <c r="G43" s="1" t="n"/>
+    </row>
+    <row r="44" ht="14" customHeight="1">
+      <c r="A44" s="20" t="n"/>
+      <c r="B44" s="20" t="n"/>
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="20" t="n"/>
+      <c r="F44" s="20" t="n"/>
+      <c r="G44" s="20" t="n"/>
+    </row>
+    <row r="45" ht="10" customHeight="1">
+      <c r="A45" s="1" t="n"/>
+      <c r="B45" s="1" t="n"/>
+      <c r="C45" s="1" t="n"/>
+      <c r="D45" s="1" t="n"/>
+      <c r="E45" s="1" t="n"/>
+      <c r="F45" s="1" t="n"/>
+      <c r="G45" s="1" t="n"/>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>JERAHMEEL CANTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Total: 1 hr   |   Lecture: 1 hr (1 slot)   |   Laboratory: 0 hrs (0 slots)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="46" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>8:00 AM - 9:00 AM</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>SIA
+[3A]
+Room 1
+[Lecture]</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="15" t="n"/>
+      <c r="F49" s="15" t="n"/>
+      <c r="G49" s="15" t="n"/>
+    </row>
+    <row r="50" ht="46" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>9:00 AM - 10:00 AM</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="15" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="15" t="n"/>
+      <c r="F50" s="15" t="n"/>
+      <c r="G50" s="15" t="n"/>
+    </row>
+    <row r="51" ht="46" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>10:00 AM - 11:00 AM</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="n"/>
+      <c r="C51" s="15" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="15" t="n"/>
+      <c r="F51" s="15" t="n"/>
+      <c r="G51" s="15" t="n"/>
+    </row>
+    <row r="52" ht="46" customHeight="1">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>11:00 AM - 12:00 PM</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="n"/>
+      <c r="C52" s="15" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15" t="n"/>
+      <c r="G52" s="15" t="n"/>
+    </row>
+    <row r="53" ht="46" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="n"/>
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="15" t="n"/>
+      <c r="F53" s="15" t="n"/>
+      <c r="G53" s="15" t="n"/>
+    </row>
+    <row r="54" ht="46" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>1:00 PM - 2:00 PM</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="n"/>
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="15" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="15" t="n"/>
+    </row>
+    <row r="55" ht="46" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>2:00 PM - 3:00 PM</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="n"/>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="15" t="n"/>
+      <c r="F55" s="15" t="n"/>
+      <c r="G55" s="15" t="n"/>
+    </row>
+    <row r="56" ht="46" customHeight="1">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>3:00 PM - 4:00 PM</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="n"/>
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+      <c r="F56" s="15" t="n"/>
+      <c r="G56" s="15" t="n"/>
+    </row>
+    <row r="57" ht="46" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>4:00 PM - 5:00 PM</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="n"/>
+      <c r="C57" s="15" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="15" t="n"/>
+      <c r="F57" s="15" t="n"/>
+      <c r="G57" s="15" t="n"/>
+    </row>
+    <row r="58" ht="46" customHeight="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>5:00 PM - 6:00 PM</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="n"/>
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="15" t="n"/>
+      <c r="F58" s="15" t="n"/>
+      <c r="G58" s="15" t="n"/>
+    </row>
+    <row r="59" ht="46" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="n"/>
+      <c r="C59" s="15" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="15" t="n"/>
+      <c r="F59" s="15" t="n"/>
+      <c r="G59" s="15" t="n"/>
+    </row>
+    <row r="60" ht="46" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>7:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="n"/>
+      <c r="C60" s="15" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="15" t="n"/>
+      <c r="F60" s="15" t="n"/>
+      <c r="G60" s="15" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Laboratory</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lecture Room</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="n"/>
+      <c r="E61" s="1" t="n"/>
+      <c r="F61" s="1" t="n"/>
+      <c r="G61" s="1" t="n"/>
+    </row>
+    <row r="62" ht="14" customHeight="1">
+      <c r="A62" s="20" t="n"/>
+      <c r="B62" s="20" t="n"/>
+      <c r="C62" s="20" t="n"/>
+      <c r="D62" s="20" t="n"/>
+      <c r="E62" s="20" t="n"/>
+      <c r="F62" s="20" t="n"/>
+      <c r="G62" s="20" t="n"/>
+    </row>
+    <row r="63" ht="10" customHeight="1">
+      <c r="A63" s="1" t="n"/>
+      <c r="B63" s="1" t="n"/>
+      <c r="C63" s="1" t="n"/>
+      <c r="D63" s="1" t="n"/>
+      <c r="E63" s="1" t="n"/>
+      <c r="F63" s="1" t="n"/>
+      <c r="G63" s="1" t="n"/>
+    </row>
+    <row r="64" ht="36" customHeight="1">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>JUAN DELA CRUZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Total: 3 hrs   |   Lecture: 2 hrs (1 slot)   |   Laboratory: 1 hr (1 slot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="24" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="46" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>8:00 AM - 9:00 AM</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>Programming
+[BSIT 3A]
+Room 2
+[Lecture]</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="15" t="n"/>
+      <c r="F67" s="15" t="n"/>
+      <c r="G67" s="15" t="n"/>
+    </row>
+    <row r="68" ht="46" customHeight="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>9:00 AM - 10:00 AM</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Programming
+[BSIT 3A]
+Room 2
+[Lecture]</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="15" t="n"/>
+      <c r="F68" s="15" t="n"/>
+      <c r="G68" s="15" t="n"/>
+    </row>
+    <row r="69" ht="46" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>10:00 AM - 11:00 AM</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="n"/>
+      <c r="C69" s="15" t="n"/>
+      <c r="D69" s="15" t="n"/>
+      <c r="E69" s="15" t="n"/>
+      <c r="F69" s="15" t="n"/>
+      <c r="G69" s="15" t="n"/>
+    </row>
+    <row r="70" ht="46" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>11:00 AM - 12:00 PM</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="15" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="15" t="n"/>
+      <c r="F70" s="15" t="n"/>
+      <c r="G70" s="15" t="n"/>
+    </row>
+    <row r="71" ht="46" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="15" t="n"/>
+      <c r="D71" s="15" t="n"/>
+      <c r="E71" s="15" t="n"/>
+      <c r="F71" s="15" t="n"/>
+      <c r="G71" s="15" t="n"/>
+    </row>
+    <row r="72" ht="46" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>1:00 PM - 2:00 PM</t>
+        </is>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>Database Management
+[BSIT 3B]
+Lab A
+[Laboratory]</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="n"/>
+      <c r="D72" s="15" t="n"/>
+      <c r="E72" s="15" t="n"/>
+      <c r="F72" s="15" t="n"/>
+      <c r="G72" s="15" t="n"/>
+    </row>
+    <row r="73" ht="46" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>2:00 PM - 3:00 PM</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="n"/>
+      <c r="C73" s="15" t="n"/>
+      <c r="D73" s="15" t="n"/>
+      <c r="E73" s="15" t="n"/>
+      <c r="F73" s="15" t="n"/>
+      <c r="G73" s="15" t="n"/>
+    </row>
+    <row r="74" ht="46" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>3:00 PM - 4:00 PM</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="n"/>
+      <c r="C74" s="15" t="n"/>
+      <c r="D74" s="15" t="n"/>
+      <c r="E74" s="15" t="n"/>
+      <c r="F74" s="15" t="n"/>
+      <c r="G74" s="15" t="n"/>
+    </row>
+    <row r="75" ht="46" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>4:00 PM - 5:00 PM</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="n"/>
+      <c r="C75" s="15" t="n"/>
+      <c r="D75" s="15" t="n"/>
+      <c r="E75" s="15" t="n"/>
+      <c r="F75" s="15" t="n"/>
+      <c r="G75" s="15" t="n"/>
+    </row>
+    <row r="76" ht="46" customHeight="1">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>5:00 PM - 6:00 PM</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="n"/>
+      <c r="C76" s="15" t="n"/>
+      <c r="D76" s="15" t="n"/>
+      <c r="E76" s="15" t="n"/>
+      <c r="F76" s="15" t="n"/>
+      <c r="G76" s="15" t="n"/>
+    </row>
+    <row r="77" ht="46" customHeight="1">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="n"/>
+      <c r="C77" s="15" t="n"/>
+      <c r="D77" s="15" t="n"/>
+      <c r="E77" s="15" t="n"/>
+      <c r="F77" s="15" t="n"/>
+      <c r="G77" s="15" t="n"/>
+    </row>
+    <row r="78" ht="46" customHeight="1">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>7:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="B78" s="15" t="n"/>
+      <c r="C78" s="15" t="n"/>
+      <c r="D78" s="15" t="n"/>
+      <c r="E78" s="15" t="n"/>
+      <c r="F78" s="15" t="n"/>
+      <c r="G78" s="15" t="n"/>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Laboratory</t>
+        </is>
+      </c>
+      <c r="C79" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lecture Room</t>
+        </is>
+      </c>
+      <c r="D79" s="1" t="n"/>
+      <c r="E79" s="1" t="n"/>
+      <c r="F79" s="1" t="n"/>
+      <c r="G79" s="1" t="n"/>
+    </row>
+    <row r="80" ht="14" customHeight="1">
+      <c r="A80" s="20" t="n"/>
+      <c r="B80" s="20" t="n"/>
+      <c r="C80" s="20" t="n"/>
+      <c r="D80" s="20" t="n"/>
+      <c r="E80" s="20" t="n"/>
+      <c r="F80" s="20" t="n"/>
+      <c r="G80" s="20" t="n"/>
+    </row>
+    <row r="81" ht="10" customHeight="1">
+      <c r="A81" s="1" t="n"/>
+      <c r="B81" s="1" t="n"/>
+      <c r="C81" s="1" t="n"/>
+      <c r="D81" s="1" t="n"/>
+      <c r="E81" s="1" t="n"/>
+      <c r="F81" s="1" t="n"/>
+      <c r="G81" s="1" t="n"/>
+    </row>
+    <row r="82" ht="36" customHeight="1">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>HELLO WORLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Total: 1 hr   |   Lecture: 1 hr (1 slot)   |   Laboratory: 0 hrs (0 slots)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="24" customHeight="1">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E84" s="12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="F84" s="12" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G84" s="12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="46" customHeight="1">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>8:00 AM - 9:00 AM</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>IT Era
+[1D]
+Room 5
+[Lecture]</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="n"/>
+      <c r="D85" s="15" t="n"/>
+      <c r="E85" s="15" t="n"/>
+      <c r="F85" s="15" t="n"/>
+      <c r="G85" s="15" t="n"/>
+    </row>
+    <row r="86" ht="46" customHeight="1">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>9:00 AM - 10:00 AM</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="n"/>
+      <c r="C86" s="15" t="n"/>
+      <c r="D86" s="15" t="n"/>
+      <c r="E86" s="15" t="n"/>
+      <c r="F86" s="15" t="n"/>
+      <c r="G86" s="15" t="n"/>
+    </row>
+    <row r="87" ht="46" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>10:00 AM - 11:00 AM</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="n"/>
+      <c r="C87" s="15" t="n"/>
+      <c r="D87" s="15" t="n"/>
+      <c r="E87" s="15" t="n"/>
+      <c r="F87" s="15" t="n"/>
+      <c r="G87" s="15" t="n"/>
+    </row>
+    <row r="88" ht="46" customHeight="1">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>11:00 AM - 12:00 PM</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="n"/>
+      <c r="C88" s="15" t="n"/>
+      <c r="D88" s="15" t="n"/>
+      <c r="E88" s="15" t="n"/>
+      <c r="F88" s="15" t="n"/>
+      <c r="G88" s="15" t="n"/>
+    </row>
+    <row r="89" ht="46" customHeight="1">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="n"/>
+      <c r="C89" s="15" t="n"/>
+      <c r="D89" s="15" t="n"/>
+      <c r="E89" s="15" t="n"/>
+      <c r="F89" s="15" t="n"/>
+      <c r="G89" s="15" t="n"/>
+    </row>
+    <row r="90" ht="46" customHeight="1">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>1:00 PM - 2:00 PM</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="n"/>
+      <c r="C90" s="15" t="n"/>
+      <c r="D90" s="15" t="n"/>
+      <c r="E90" s="15" t="n"/>
+      <c r="F90" s="15" t="n"/>
+      <c r="G90" s="15" t="n"/>
+    </row>
+    <row r="91" ht="46" customHeight="1">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>2:00 PM - 3:00 PM</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="n"/>
+      <c r="C91" s="15" t="n"/>
+      <c r="D91" s="15" t="n"/>
+      <c r="E91" s="15" t="n"/>
+      <c r="F91" s="15" t="n"/>
+      <c r="G91" s="15" t="n"/>
+    </row>
+    <row r="92" ht="46" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>3:00 PM - 4:00 PM</t>
+        </is>
+      </c>
+      <c r="B92" s="15" t="n"/>
+      <c r="C92" s="15" t="n"/>
+      <c r="D92" s="15" t="n"/>
+      <c r="E92" s="15" t="n"/>
+      <c r="F92" s="15" t="n"/>
+      <c r="G92" s="15" t="n"/>
+    </row>
+    <row r="93" ht="46" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>4:00 PM - 5:00 PM</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="n"/>
+      <c r="C93" s="15" t="n"/>
+      <c r="D93" s="15" t="n"/>
+      <c r="E93" s="15" t="n"/>
+      <c r="F93" s="15" t="n"/>
+      <c r="G93" s="15" t="n"/>
+    </row>
+    <row r="94" ht="46" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>5:00 PM - 6:00 PM</t>
+        </is>
+      </c>
+      <c r="B94" s="15" t="n"/>
+      <c r="C94" s="15" t="n"/>
+      <c r="D94" s="15" t="n"/>
+      <c r="E94" s="15" t="n"/>
+      <c r="F94" s="15" t="n"/>
+      <c r="G94" s="15" t="n"/>
+    </row>
+    <row r="95" ht="46" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="n"/>
+      <c r="C95" s="15" t="n"/>
+      <c r="D95" s="15" t="n"/>
+      <c r="E95" s="15" t="n"/>
+      <c r="F95" s="15" t="n"/>
+      <c r="G95" s="15" t="n"/>
+    </row>
+    <row r="96" ht="46" customHeight="1">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>7:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="n"/>
+      <c r="C96" s="15" t="n"/>
+      <c r="D96" s="15" t="n"/>
+      <c r="E96" s="15" t="n"/>
+      <c r="F96" s="15" t="n"/>
+      <c r="G96" s="15" t="n"/>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="17" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Laboratory</t>
+        </is>
+      </c>
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lecture Room</t>
+        </is>
+      </c>
+      <c r="D97" s="1" t="n"/>
+      <c r="E97" s="1" t="n"/>
+      <c r="F97" s="1" t="n"/>
+      <c r="G97" s="1" t="n"/>
+    </row>
+    <row r="98" ht="14" customHeight="1">
+      <c r="A98" s="20" t="n"/>
+      <c r="B98" s="20" t="n"/>
+      <c r="C98" s="20" t="n"/>
+      <c r="D98" s="20" t="n"/>
+      <c r="E98" s="20" t="n"/>
+      <c r="F98" s="20" t="n"/>
+      <c r="G98" s="20" t="n"/>
+    </row>
+    <row r="99" ht="10" customHeight="1">
+      <c r="A99" s="1" t="n"/>
+      <c r="B99" s="1" t="n"/>
+      <c r="C99" s="1" t="n"/>
+      <c r="D99" s="1" t="n"/>
+      <c r="E99" s="1" t="n"/>
+      <c r="F99" s="1" t="n"/>
+      <c r="G99" s="1" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="15">
     <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A83:G83"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A82:G82"/>
+    <mergeCell ref="A65:G65"/>
     <mergeCell ref="A11:G11"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>

</xml_diff>